<commit_message>
sensi analysis + plein de trucs
</commit_message>
<xml_diff>
--- a/courbes/summary_table.xlsx
+++ b/courbes/summary_table.xlsx
@@ -591,57 +591,57 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>20/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>0.7106</t>
+          <t>0.7124</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>52/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>0.7096</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>126/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>0.7050</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>236/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>0.7009</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>CMApara</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>0.7119</t>
+          <t>0.7126</t>
         </is>
       </c>
     </row>
@@ -663,57 +663,57 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>13/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>0.7429</t>
+          <t>0.7471</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>57/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>0.7391</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>146/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>0.7317</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>204/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>0.7274</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>CMApara</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>0.7459</t>
+          <t>0.7497</t>
         </is>
       </c>
     </row>
@@ -735,58 +735,57 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>21/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>0.7504</t>
+          <t>0.7606</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>40/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>0.7463</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>146/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>0.7330</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>179/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>0.7311</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>ChainCMAwithMetaRe
-centeringsqrt</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>0.7565</t>
+          <t>0.7658</t>
         </is>
       </c>
     </row>
@@ -808,58 +807,57 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>14/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>0.7396</t>
+          <t>0.7565</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>34/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>0.7330</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>262/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>0.7088</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>308/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>0.6932</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>ChainCMAwithLHSsqr
-t</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>0.7493</t>
+          <t>0.7535</t>
         </is>
       </c>
     </row>
@@ -881,57 +879,57 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>0.7098</t>
+          <t>0.7119</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>4/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>0.7061</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>158/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>0.6959</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>206/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>0.6941</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>CMApara</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>0.7075</t>
+          <t>0.7094</t>
         </is>
       </c>
     </row>
@@ -953,57 +951,57 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>0.7344</t>
+          <t>0.7410</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>0.7305</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>140/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>0.7138</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>138/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>0.7139</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>CMApara</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>3/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>0.7304</t>
+          <t>0.7364</t>
         </is>
       </c>
     </row>
@@ -1025,57 +1023,57 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>0.7555</t>
+          <t>0.7665</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>0.7465</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>202/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>0.7191</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>124/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>0.7252</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>MetaModelFmin2</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>3/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>0.7431</t>
+          <t>0.7535</t>
         </is>
       </c>
     </row>
@@ -1097,57 +1095,57 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>0.7353</t>
+          <t>0.7436</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>0.7266</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>355/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>0.6372</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>387/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>0.6071</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>CMAL3</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>3/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>0.7256</t>
+          <t>0.7373</t>
         </is>
       </c>
     </row>
@@ -1169,57 +1167,57 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>0.7072</t>
+          <t>0.7092</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>0.7014</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>111/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>0.6810</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>87/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>0.6869</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>CMApara</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>3/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>0.6989</t>
+          <t>0.7029</t>
         </is>
       </c>
     </row>
@@ -1241,57 +1239,58 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>0.7343</t>
+          <t>0.7403</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>0.7249</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>98/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>0.7004</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>60/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>0.7100</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>MetaModelFmin2</t>
+          <t>HugeLognormalDiscr
+eteOnePlusOne</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>3/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>0.7218</t>
+          <t>0.7269</t>
         </is>
       </c>
     </row>
@@ -1313,57 +1312,58 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>0.7477</t>
+          <t>0.7587</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>0.7336</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>104/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>0.7007</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>179/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>0.6895</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>MetaModelFmin2</t>
+          <t>HugeLognormalDiscr
+eteOnePlusOne</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>3/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>0.7295</t>
+          <t>0.7352</t>
         </is>
       </c>
     </row>
@@ -1385,58 +1385,59 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>0.7248</t>
+          <t>0.7290</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>0.7171</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>384/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>0.5798</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>389/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>0.5730</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>LognormalDiscreteO
-nePlusOne</t>
+          <t>OnePtRecombiningDi
+screteLenglerOnePl
+usOne</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>3/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>0.7166</t>
+          <t>0.7242</t>
         </is>
       </c>
     </row>
@@ -1458,57 +1459,57 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>102/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>-198.2</t>
+          <t>205.5</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>60/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>-199.8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>249/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>-188.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>267/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>-184.6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>CMAL3</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>-206.2</t>
+          <t>212.2</t>
         </is>
       </c>
     </row>
@@ -1530,57 +1531,57 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>140/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>-145.3</t>
+          <t>151.9</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>90/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>-147.8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>133/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>-146.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>139/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>-145.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>CMApara</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>-154.3</t>
+          <t>154.6</t>
         </is>
       </c>
     </row>
@@ -1602,42 +1603,42 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>164/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>-137.1</t>
+          <t>142.2</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>88/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>-139.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>118/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>-137.6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>153/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>-137.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1647,12 +1648,12 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>-143.4</t>
+          <t>144.7</t>
         </is>
       </c>
     </row>
@@ -1674,57 +1675,57 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>79/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>-411.1</t>
+          <t>429.0</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>89/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>-410.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>264/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>-379.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>266/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>-377.5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>ChainCMAwithRsqrt</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>-430.7</t>
+          <t>445.3</t>
         </is>
       </c>
     </row>
@@ -1746,57 +1747,57 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>129/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>-323.6</t>
+          <t>338.6</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>80/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>-329.7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>264/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>-311.7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>275/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>-309.7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>CMApara</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>-344.2</t>
+          <t>345.5</t>
         </is>
       </c>
     </row>
@@ -1818,57 +1819,57 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>137/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>-304.4</t>
+          <t>316.4</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>65/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>-310.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>241/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>-298.3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>260/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>-295.9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>CMApara</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>-319.3</t>
+          <t>326.1</t>
         </is>
       </c>
     </row>
@@ -1890,58 +1891,57 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>46/503</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>-577.1</t>
+          <t>601.0</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>64/503</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>-570.8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>255/503</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>-504.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>223/503</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>-517.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>DiscreteLengler2On
-ePlusOne</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>1/503</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>-587.7</t>
+          <t>616.4</t>
         </is>
       </c>
     </row>
@@ -1963,57 +1963,57 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>30/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>-436.5</t>
+          <t>451.1</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>20/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>-438.3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>241/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>-408.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>226/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>-413.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>CMApara</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>-453.8</t>
+          <t>465.8</t>
         </is>
       </c>
     </row>
@@ -2035,57 +2035,57 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>29/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>-425.0</t>
+          <t>438.4</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>18/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>-427.5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>237/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>-398.9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>222/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>-403.7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>CMAL3</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>-435.4</t>
+          <t>451.9</t>
         </is>
       </c>
     </row>
@@ -2107,57 +2107,57 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>47/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>-1193.3</t>
+          <t>1232.9</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>78/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>-1177.9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>257/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>-1034.7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>253/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>-1046.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>NgIoh</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>-1207.2</t>
+          <t>1280.2</t>
         </is>
       </c>
     </row>
@@ -2179,57 +2179,57 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>19/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>-932.9</t>
+          <t>964.8</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>16/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>-934.5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>265/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>-842.8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>253/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>-857.3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>CMApara</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>-964.9</t>
+          <t>994.7</t>
         </is>
       </c>
     </row>
@@ -2251,57 +2251,57 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>19/504</t>
+          <t>3/80</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>-912.6</t>
+          <t>937.6</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>53/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>-907.6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>263/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>-817.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>249/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>-830.9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>CMAL3</t>
+          <t>DiscreteDE</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>-928.6</t>
+          <t>967.3</t>
         </is>
       </c>
     </row>
@@ -2323,57 +2323,58 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>27/80</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>-1623.5</t>
+          <t>1671.7</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>46/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>-1570.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>199/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>-1317.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>99/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>-1422.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>NLOPT_LN_PRAXIS</t>
+          <t>DiscreteLengler3On
+ePlusOne</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>-1607.1</t>
+          <t>1694.5</t>
         </is>
       </c>
     </row>
@@ -2395,58 +2396,58 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>-1300.4</t>
+          <t>1340.8</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>3/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>-1290.5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>197/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>-1105.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>92/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>-1197.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>BigLognormalDiscre
-teOnePlusOne</t>
+          <t>HugeLognormalDiscr
+eteOnePlusOne</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>2/80</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>-1301.4</t>
+          <t>1340.1</t>
         </is>
       </c>
     </row>
@@ -2468,58 +2469,58 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>22/80</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>-1234.7</t>
+          <t>1264.0</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>12/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>-1230.9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>187/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>-1073.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>92/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>-1154.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>SVMMetaModelLogNor
-mal</t>
+          <t>DiscreteLengler3On
+ePlusOne</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>-1233.8</t>
+          <t>1293.5</t>
         </is>
       </c>
     </row>
@@ -2541,57 +2542,58 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>3/504</t>
+          <t>40/80</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>-3285.9</t>
+          <t>3376.6</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>53/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>-3208.6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>196/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>-2650.7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>148/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>-2854.3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>RLSOnePlusOne</t>
+          <t>DiscreteLengler3On
+ePlusOne</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>-3316.5</t>
+          <t>3453.3</t>
         </is>
       </c>
     </row>
@@ -2613,58 +2615,58 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>3/80</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>-2633.4</t>
+          <t>2706.1</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>35/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>-2597.5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>208/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>-2219.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>134/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>-2391.5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>DiscreteLengler2On
-ePlusOne</t>
+          <t>HugeLognormalDiscr
+eteOnePlusOne</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>-2617.0</t>
+          <t>2717.2</t>
         </is>
       </c>
     </row>
@@ -2686,58 +2688,58 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>1/504</t>
+          <t>12/80</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>-2606.9</t>
+          <t>2672.3</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>41/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>-2557.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>185/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>-2206.6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>141/504</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>-2349.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>SVM1MetaModelLogNo
-rmal</t>
+          <t>HugeLognormalDiscr
+eteOnePlusOne</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>2/504</t>
+          <t>1/80</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>-2605.1</t>
+          <t>2712.2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ajout des eda classique
</commit_message>
<xml_diff>
--- a/courbes/summary_table.xlsx
+++ b/courbes/summary_table.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -601,32 +601,32 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>36/83</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7097</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7052</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7008</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -673,32 +673,32 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10/83</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7412</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>53/83</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7312</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7262</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -745,32 +745,32 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4/83</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7492</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7330</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>55/83</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7316</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -817,32 +817,32 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8/83</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7368</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7176</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>55/83</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7174</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -889,32 +889,32 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7085</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.6956</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.6928</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -961,32 +961,32 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7334</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>55/83</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7147</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7135</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1033,32 +1033,32 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7514</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7229</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>53/83</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7285</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1105,32 +1105,32 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7369</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>55/83</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7034</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.6681</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1177,32 +1177,32 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7048</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.6802</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>50/83</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.6863</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1249,32 +1249,32 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7314</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.6989</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>48/83</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7093</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1322,32 +1322,32 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7429</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>55/83</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7019</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>47/83</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7162</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1395,32 +1395,32 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7315</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>55/83</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.6805</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>62/83</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5852</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>0.7322</t>
+          <t>0.7321</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>0.7243</t>
+          <t>0.7238</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>0.7246</t>
+          <t>0.7249</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2215,12 +2215,12 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>56/83</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>0.7064</t>
+          <t>0.7072</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>0.5798</t>
+          <t>0.5790</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2341,32 +2341,32 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>24/83</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>200.7</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>57/83</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>187.9</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>59/83</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>184.2</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2413,32 +2413,32 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5/83</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>149.7</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>25/83</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>145.7</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>46/83</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>144.3</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>3/80</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2485,32 +2485,32 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13/83</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>139.6</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>46/83</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>137.5</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>45/83</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>137.5</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -2520,7 +2520,7 @@
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2557,32 +2557,32 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>36/83</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>412.8</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>59/83</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>375.6</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>58/83</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>379.7</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2629,32 +2629,32 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5/83</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>330.2</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>57/83</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>313.7</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>313.8</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2701,32 +2701,32 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>19/83</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>310.6</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>297.3</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>58/83</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>296.7</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2773,32 +2773,32 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>18/83</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>585.8</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>505.2</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>511.8</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2845,32 +2845,32 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4/83</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>445.5</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>55/83</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>410.9</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>412.6</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>3/80</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2917,32 +2917,32 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11/83</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>430.5</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>402.5</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>405.8</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>4/80</t>
+          <t>4/83</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2989,32 +2989,32 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15/83</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1211.7</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>57/83</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1030.1</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1048.9</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>3/80</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -3061,32 +3061,32 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7/83</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>936.2</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>841.7</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>55/83</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>865.7</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>3/80</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -3133,32 +3133,32 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10/83</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>928.4</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>818.9</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>829.0</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>34/80</t>
+          <t>35/83</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -3205,32 +3205,32 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>16/83</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1680.4</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1327.4</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>53/83</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1418.7</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
@@ -3268,7 +3268,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -3278,32 +3278,32 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7/83</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1322.3</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1102.8</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>51/83</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1191.6</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>2/80</t>
+          <t>2/83</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
@@ -3341,7 +3341,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>12/80</t>
+          <t>13/83</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -3351,32 +3351,32 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11/83</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1277.8</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1085.0</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>51/83</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1146.9</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>40/80</t>
+          <t>41/83</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -3424,32 +3424,32 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>29/83</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3406.7</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>57/83</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2646.0</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2881.9</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>3/80</t>
+          <t>3/83</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -3497,32 +3497,32 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7/83</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2656.3</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>56/83</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2245.8</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>54/83</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2399.2</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>38/80</t>
+          <t>39/83</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -3570,32 +3570,32 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7/83</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2681.7</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>57/83</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2177.0</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>53/83</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2362.4</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>1/80</t>
+          <t>1/83</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">

</xml_diff>